<commit_message>
Show survey instructions only on the first chained part
English_Word_Ratings_2 and _3 were repeating the same instructions page
as part 1, even though all three parts are chained into one formr run --
participants only need to see it once. make_template() now takes
instructions_label = NULL to skip that intro block entirely; English's
make_template.R only supplies it for part 1. Regenerated templates,
rebuilt the live xlsx files, and pushed the fix to formr.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-Task/English/English_Word_Ratings.xlsx
+++ b/02-Task/English/English_Word_Ratings.xlsx
@@ -108,8 +108,8 @@
     <t xml:space="preserve">w01_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **lightning**
- Please name all of the ways someone could use a **lightning**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **songbird**
+ Please name all of the ways someone could use a **songbird**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">01</t>
@@ -247,8 +247,8 @@
     <t xml:space="preserve">w02_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **sarcophagus**
- Please name all of the ways someone could use a **sarcophagus**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **bucktooth**
+ Please name all of the ways someone could use a **bucktooth**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">02</t>
@@ -296,8 +296,8 @@
     <t xml:space="preserve">w03_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **salon**
- Please name all of the ways someone could use a **salon**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **centrifuge**
+ Please name all of the ways someone could use a **centrifuge**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">03</t>
@@ -345,8 +345,8 @@
     <t xml:space="preserve">w04_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **watchtower**
- Please name all of the ways someone could use a **watchtower**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **town**
+ Please name all of the ways someone could use a **town**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">04</t>
@@ -394,8 +394,8 @@
     <t xml:space="preserve">w05_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **trident**
- Please name all of the ways someone could use a **trident**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **omelette**
+ Please name all of the ways someone could use a **omelette**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">05</t>
@@ -443,8 +443,8 @@
     <t xml:space="preserve">w06_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **flintstone**
- Please name all of the ways someone could use a **flintstone**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **orangutan**
+ Please name all of the ways someone could use a **orangutan**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">06</t>
@@ -492,8 +492,8 @@
     <t xml:space="preserve">w07_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **brig**
- Please name all of the ways someone could use a **brig**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **cub**
+ Please name all of the ways someone could use a **cub**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">07</t>
@@ -541,8 +541,8 @@
     <t xml:space="preserve">w08_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **park**
- Please name all of the ways someone could use a **park**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **millimeter**
+ Please name all of the ways someone could use a **millimeter**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">08</t>
@@ -590,8 +590,8 @@
     <t xml:space="preserve">w09_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **sloth**
- Please name all of the ways someone could use a **sloth**. Put one different use in each sloth.</t>
+    <t xml:space="preserve">### Word: **mansions**
+ Please name all of the ways someone could use a **mansions**. Put one different use in each mansions.</t>
   </si>
   <si>
     <t xml:space="preserve">09</t>
@@ -639,8 +639,8 @@
     <t xml:space="preserve">w10_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **excrement**
- Please name all of the ways someone could use a **excrement**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **firelight**
+ Please name all of the ways someone could use a **firelight**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">w10_use_01</t>

</xml_diff>

<commit_message>
Bias word selection toward the 500-word cross-linguistic overlap set
select_words() now takes an optional priority_cues argument: undersampled
priority cues fill as many of each build's slots as they can (still
inverse-N weighted within that set, not a fixed order) before falling
back to the general pool. English's build_formr_xlsx.R wires this to
01-Stimuli/shared_core_top500.csv via the new priority_words.R, which
loads gloss_english directly for English (the gloss language that file
is built around) but will need to extract each other language's own
translation of those 500 concepts from that file's words column once
they come online -- their priority set is only as large as their own
translation coverage, not assumed to be all 500.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-Task/English/English_Word_Ratings.xlsx
+++ b/02-Task/English/English_Word_Ratings.xlsx
@@ -108,8 +108,8 @@
     <t xml:space="preserve">w01_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **songbird**
- Please name all of the ways someone could use a **songbird**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **jewel**
+ Please name all of the ways someone could use a **jewel**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">01</t>
@@ -247,8 +247,8 @@
     <t xml:space="preserve">w02_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **bucktooth**
- Please name all of the ways someone could use a **bucktooth**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **crowd**
+ Please name all of the ways someone could use a **crowd**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">02</t>
@@ -296,8 +296,8 @@
     <t xml:space="preserve">w03_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **centrifuge**
- Please name all of the ways someone could use a **centrifuge**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **airport**
+ Please name all of the ways someone could use a **airport**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">03</t>
@@ -343,159 +343,159 @@
   </si>
   <si>
     <t xml:space="preserve">w04_prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">### Word: **president**
+ Please name all of the ways someone could use a **president**. Put one different use in each box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_more</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_more == 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_use_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w04_submit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">### Word: **monkey**
+ Please name all of the ways someone could use a **monkey**. Put one different use in each box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_more</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_more == 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_use_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w05_submit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">### Word: **crack**
+ Please name all of the ways someone could use a **crack**. Put one different use in each box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_more</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_more == 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_use_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w06_submit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w07_prompt</t>
   </si>
   <si>
     <t xml:space="preserve">### Word: **town**
  Please name all of the ways someone could use a **town**. Put one different use in each box.</t>
   </si>
   <si>
-    <t xml:space="preserve">04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_more</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_more == 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_use_10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w04_submit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_prompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">### Word: **omelette**
- Please name all of the ways someone could use a **omelette**. Put one different use in each box.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_more</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_more == 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_use_10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w05_submit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_prompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">### Word: **orangutan**
- Please name all of the ways someone could use a **orangutan**. Put one different use in each box.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_more</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_more == 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_use_10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w06_submit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">w07_prompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">### Word: **cub**
- Please name all of the ways someone could use a **cub**. Put one different use in each box.</t>
-  </si>
-  <si>
     <t xml:space="preserve">07</t>
   </si>
   <si>
@@ -541,8 +541,8 @@
     <t xml:space="preserve">w08_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **millimeter**
- Please name all of the ways someone could use a **millimeter**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **room**
+ Please name all of the ways someone could use a **room**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">08</t>
@@ -590,8 +590,8 @@
     <t xml:space="preserve">w09_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **mansions**
- Please name all of the ways someone could use a **mansions**. Put one different use in each mansions.</t>
+    <t xml:space="preserve">### Word: **blackbird**
+ Please name all of the ways someone could use a **blackbird**. Put one different use in each blackbird.</t>
   </si>
   <si>
     <t xml:space="preserve">09</t>
@@ -639,8 +639,8 @@
     <t xml:space="preserve">w10_prompt</t>
   </si>
   <si>
-    <t xml:space="preserve">### Word: **firelight**
- Please name all of the ways someone could use a **firelight**. Put one different use in each box.</t>
+    <t xml:space="preserve">### Word: **fat**
+ Please name all of the ways someone could use a **fat**. Put one different use in each box.</t>
   </si>
   <si>
     <t xml:space="preserve">w10_use_01</t>

</xml_diff>